<commit_message>
Crossdock Master Setting: apply business decisions (FSD v0.3)
- Effective Start Date editable only while the part is still Candidate (BR-06)
- Keep the Edit button on the Part List row next to the Part Number link (BR-07)
- FSD: ongoing period lists Active parts, past periods list every part (BR-12)
- FSD: "Validate file" is the save button after upload (OP-02)
- FSD: mapping total below or equal to Max Case/Day is allowed (BR-16, OP-04)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/FSD_Crossdock_Master_Setting.xlsx
+++ b/FSD_Crossdock_Master_Setting.xlsx
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>0.2 (Draft)</t>
+          <t xml:space="preserve">0.3 (Draft)</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1981,6 +1981,23 @@
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="62" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.3</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Business decisions: Effective Start Date editable only while Candidate (BR-06 confirmed); Edit button kept next to the Part Number link (BR-07); ongoing period lists Active parts, past periods list every part (BR-12); "Validate file" = save after upload (OP-02); allocation below or equal to Max Case/Day allowed (BR-16, OP-04).</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2537,7 @@
     <row r="34" ht="71" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>In the prototype "Validate file" only closes the modal; the validation flow and error messages are not defined yet.</t>
+          <t xml:space="preserve">"Validate file" is the save button after upload: it validates the file and saves the data when every row is valid; otherwise nothing is saved. In the prototype it only closes the modal; the detailed validation rules and messages are in FSD Crossdock Upload Batch.</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr"/>
@@ -2637,12 +2654,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>The Export Excel button in the Part List header has no action. Upload Excel: "Validate file" only closes the modal; there is no validation flow, error message or result.</t>
+          <t xml:space="preserve">The Export Excel button in the Part List header has no action. Upload Excel: "Validate file" only closes the modal in the prototype.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Define the content of the Part List export (used as the base file for Edit uploads) and the upload validation flow with its error messages.</t>
+          <t xml:space="preserve">DECIDED (v0.3): "Validate file" is the save button after upload — it validates the uploaded file and saves it (all-or-nothing). Validation rules and messages: FSD Crossdock Upload Batch. Still open: content of the Part List export used as the base file for Edit uploads.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2696,7 +2713,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Confirm whether the allocation must equal Max Case/Day exactly, and reject rows without a destination.</t>
+          <t xml:space="preserve">DECIDED (v0.3): the total Case/Day of each part must not exceed its Max Case/Day; a total below or equal to Max Case/Day is allowed. Still open: whether rows without a destination ("Select destination") are rejected.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -3309,7 +3326,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Active part. Only Active parts are shown in Mapping per Destination.</t>
+          <t xml:space="preserve">Active part. In the ongoing calculation period only Active parts are shown in Mapping per Destination.</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr"/>
@@ -3327,7 +3344,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Inactive part. Not shown in Mapping per Destination.</t>
+          <t xml:space="preserve">Inactive part. Not shown in Mapping per Destination for the ongoing period (past periods show every part, read-only).</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr"/>
@@ -4321,7 +4338,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Search PART-I and click the "Edit" button on its row.</t>
+          <t xml:space="preserve">Search PART-I and click the "Edit" button on its row (or click the Part Number link).</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -5372,7 +5389,7 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Only Active parts are listed. Only Active parts appear in the Mapping per Destination sub-menu.</t>
+          <t xml:space="preserve">Only Active parts are listed. In the ongoing period only Active parts appear in the Mapping per Destination sub-menu.</t>
         </is>
       </c>
     </row>
@@ -6948,7 +6965,7 @@
       </c>
       <c r="B219" s="5" t="inlineStr">
         <is>
-          <t>Search PART-I and click the "Edit" button on its row.</t>
+          <t xml:space="preserve">Search PART-I and click the "Edit" button on its row (or click the Part Number link; both open the same modal).</t>
         </is>
       </c>
     </row>
@@ -7306,7 +7323,7 @@
       </c>
       <c r="B346" s="5" t="inlineStr">
         <is>
-          <t>In the prototype "Validate file" only closes the modal (OP-02). Upload rules are detailed in the sheet "9 Export &amp; Upload".</t>
+          <t xml:space="preserve">"Validate file" is the save button of the upload: it validates the uploaded file and, when every row is valid, saves the data (all-or-nothing, see FSD Crossdock Upload Batch). In the prototype it only closes the modal. Upload rules are detailed in the sheet "9 Export &amp; Upload".</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8263,7 @@
     <row r="315" ht="22" customHeight="1">
       <c r="A315" s="6" t="inlineStr">
         <is>
-          <t>D10  -  Non-Active parts never appear</t>
+          <t xml:space="preserve">D10  -  Non-Active parts never appear in the ongoing period</t>
         </is>
       </c>
     </row>
@@ -8282,7 +8299,7 @@
       </c>
       <c r="B318" s="5" t="inlineStr">
         <is>
-          <t>Empty state "No parts match these filters". Mapping per Destination only lists parts with status Active, whatever the other filters are.</t>
+          <t xml:space="preserve">Empty state "No parts match these filters". In the ongoing period Mapping per Destination only lists parts with status Active, whatever the other filters are. Past periods list every part (any status), read-only.</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8645,7 @@
       </c>
       <c r="B444" s="5" t="inlineStr">
         <is>
-          <t>Rule BR-16.</t>
+          <t xml:space="preserve">Rule BR-16. Over-allocation is the only allocation that blocks Save (OP-04 decided).</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8735,7 @@
       </c>
       <c r="B479" s="5" t="inlineStr">
         <is>
-          <t>See OP-04.</t>
+          <t xml:space="preserve">Allowed: total Case/Day may be below or equal to Max Case/Day (OP-04 decided).</t>
         </is>
       </c>
     </row>
@@ -8806,7 +8823,7 @@
       </c>
       <c r="B512" s="5" t="inlineStr">
         <is>
-          <t>A row with no destination selected can still be saved (OP-04).</t>
+          <t xml:space="preserve">A row with no destination selected can still be saved (see OP-04).</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9536,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>No action yet in the prototype (OP-02).</t>
+          <t xml:space="preserve">Opens the Upload Excel modal. "Validate file" in the modal validates and saves the uploaded file (OP-02).</t>
         </is>
       </c>
     </row>
@@ -11778,7 +11795,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Part No cannot be changed when editing. Status can be changed (Candidate / Active / Inactive).</t>
+          <t xml:space="preserve">Part No cannot be changed when editing. Status can be changed (Candidate / Active / Inactive). The edit modal opens from the "Edit" button on the row and from the Part Number link; both are kept.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -11888,7 +11905,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Mapping per Destination only lists parts with status Active.</t>
+          <t xml:space="preserve">In the ongoing calculation period Mapping per Destination only lists parts with status Active. Past periods list every part (any status) and are read-only.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -11976,7 +11993,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Saving a mapping is blocked when the total Case/Day exceeds Max Case/Day or when there is no destination. A total below Max Case/Day is allowed (shown as "left").</t>
+          <t xml:space="preserve">Saving a mapping is blocked when the total Case/Day exceeds Max Case/Day or when there is no destination. A total below or equal to Max Case/Day is allowed (below is shown as "left").</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Crossdock Master Setting: block empty destination rows, upload success popup, Part List export as Edit upload base
- Mapping per Destination: Save is disabled while any row has no destination (OP-04, MSG-16)
- Upload Excel: "Validate file" saves and shows a success popup (OP-02, MSG-17)
- Part List Export Excel adds sheet "Upload" pre-filled with flag E for every part,
  in the column order of FSD Crossdock Upload Batch; sheet 1 gains Effective Start Date
- FSD v0.3 updated accordingly (BR-16, OP-02, OP-04, M11, D16, sheets 8 and 9)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/FSD_Crossdock_Master_Setting.xlsx
+++ b/FSD_Crossdock_Master_Setting.xlsx
@@ -1984,7 +1984,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="62" customHeight="1">
+    <row r="22" ht="78" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">0.3</t>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business decisions: Effective Start Date editable only while Candidate (BR-06 confirmed); Edit button kept next to the Part Number link (BR-07); ongoing period lists Active parts, past periods list every part (BR-12); "Validate file" = save after upload (OP-02); allocation below or equal to Max Case/Day allowed (BR-16, OP-04).</t>
+          <t xml:space="preserve">Business decisions: Effective Start Date editable only while Candidate (BR-06 confirmed); Edit button kept next to the Part Number link (BR-07); ongoing period lists Active parts, past periods list every part (BR-12); "Validate file" = save after upload, followed by a success popup (OP-02); Part List Export Excel sheet "Upload" is the base file for Edit uploads (OP-02); allocation below or equal to Max Case/Day allowed and every destination row must have a destination (BR-16, OP-04).</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2528,7 +2528,7 @@
     <row r="33" ht="57.8" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Edit: Export Excel must be downloaded first as the base file, then edited and uploaded again.</t>
+          <t xml:space="preserve">Edit: download the Part List Export Excel first. Its sheet "Upload" is the base file: every registered part pre-filled with its current values and flag_add_edit = E (columns part_no, minimum_mad, pcs_case, max_case_day, status, flag_add_edit, effective_start_date DD-Mon-YYYY). Sheet 1 "Part List" follows the active filter and is information only.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr"/>
@@ -2537,7 +2537,7 @@
     <row r="34" ht="71" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Validate file" is the save button after upload: it validates the file and saves the data when every row is valid; otherwise nothing is saved. In the prototype it only closes the modal; the detailed validation rules and messages are in FSD Crossdock Upload Batch.</t>
+          <t xml:space="preserve">"Validate file" is the save button after upload: it validates the file and saves the data when every row is valid; otherwise nothing is saved. After saving, the popup "Saved successfully" appears (MSG-17). Detailed validation rules and messages are in FSD Crossdock Upload Batch.</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr"/>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Export Excel button in the Part List header has no action. Upload Excel: "Validate file" only closes the modal in the prototype.</t>
+          <t xml:space="preserve">Upload Excel: "Validate file" only closed the modal; the Part List export had no defined role in the Edit upload.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECIDED (v0.3): "Validate file" is the save button after upload — it validates the uploaded file and saves it (all-or-nothing). Validation rules and messages: FSD Crossdock Upload Batch. Still open: content of the Part List export used as the base file for Edit uploads.</t>
+          <t xml:space="preserve">DECIDED (v0.3): the Part List Export Excel is the base file for Edit uploads (sheet "Upload", pre-filled with flag E). "Validate file" is the save button after upload: it validates and saves the file (all-or-nothing) and then shows a success popup. Validation rules and messages: FSD Crossdock Upload Batch.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECIDED (v0.3): the total Case/Day of each part must not exceed its Max Case/Day; a total below or equal to Max Case/Day is allowed. Still open: whether rows without a destination ("Select destination") are rejected.</t>
+          <t xml:space="preserve">DECIDED (v0.3): the total Case/Day of each part must not exceed its Max Case/Day; below or equal is allowed. A destination row without a destination cannot be saved (Save disabled, banner MSG-16).</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="B345" s="5" t="inlineStr">
         <is>
-          <t>The modal lists the template columns (flag_add_edit, part_no, pcs_case, max_case_day, minimum_mad, effective_start_date), the required columns for Add and Edit, a drag-and-drop area (.xlsx max 5 MB, max 5,000 rows), the "Download template .xlsx" link and the "Close" and "Validate file" buttons.</t>
+          <t xml:space="preserve">The modal lists the template columns (flag_add_edit, part_no, pcs_case, max_case_day, minimum_mad, effective_start_date), the required columns for Add and Edit, a drag-and-drop area (.xlsx max 5 MB, max 5,000 rows), the "Download template .xlsx" link and the "Close" and "Validate file" buttons. After "Validate file" the modal closes and the popup "Saved successfully" appears (MSG-17).</t>
         </is>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="B346" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Validate file" is the save button of the upload: it validates the uploaded file and, when every row is valid, saves the data (all-or-nothing, see FSD Crossdock Upload Batch). In the prototype it only closes the modal. Upload rules are detailed in the sheet "9 Export &amp; Upload".</t>
+          <t xml:space="preserve">"Validate file" is the save button of the upload: it validates the uploaded file and, when every row is valid, saves the data (all-or-nothing, see FSD Crossdock Upload Batch), then shows the success popup (MSG-17). The base file for Edit rows is sheet "Upload" of the Part List Export Excel. In the prototype the file is not read, so the Part List does not change.</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="B512" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A row with no destination selected can still be saved (see OP-04).</t>
+          <t xml:space="preserve">Save is disabled while any row has no destination selected; the banner MSG-16 is shown (OP-04 decided).</t>
         </is>
       </c>
     </row>
@@ -9536,7 +9536,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opens the Upload Excel modal. "Validate file" in the modal validates and saves the uploaded file (OP-02).</t>
+          <t xml:space="preserve">Opens the Upload Excel modal. "Validate file" in the modal validates and saves the uploaded file, then shows the success popup (OP-02).</t>
         </is>
       </c>
     </row>
@@ -11993,7 +11993,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saving a mapping is blocked when the total Case/Day exceeds Max Case/Day or when there is no destination. A total below or equal to Max Case/Day is allowed (below is shown as "left").</t>
+          <t xml:space="preserve">Saving a mapping is blocked when the total Case/Day exceeds Max Case/Day, when there is no destination, or when any destination row has no destination selected. A total below or equal to Max Case/Day is allowed (below is shown as "left").</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -12062,7 +12062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12437,6 +12437,50 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="31.4" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MSG-16</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mapping - row without destination</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select a destination for every row, or remove the empty row, before saving.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edit mode, at least one row still shows "Select destination". Save is disabled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="31.4" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MSG-17</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upload Excel - success popup</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved successfully — "Upload completed. The file has been validated and the part settings have been saved to the Part List." [OK]</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After "Validate file" in the Upload Excel modal.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>

</xml_diff>

<commit_message>
Upload template: add status column, Candidate status cannot be changed by upload
- Upload Excel modal lists the 7 columns of sheet "Upload" in the same order and
  states the status rule: Candidate stays Candidate, Active <-> Inactive allowed,
  nothing can become Candidate
- FSD Crossdock Master Setting v0.3: upload template table and M11 updated
- FSD Crossdock Upload Batch v0.2: template (status), PR-03 and PL-09 updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/FSD_Crossdock_Master_Setting.xlsx
+++ b/FSD_Crossdock_Master_Setting.xlsx
@@ -1984,7 +1984,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="78" customHeight="1">
+    <row r="22" ht="92" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">0.3</t>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business decisions: Effective Start Date editable only while Candidate (BR-06 confirmed); Edit button kept next to the Part Number link (BR-07); ongoing period lists Active parts, past periods list every part (BR-12); "Validate file" = save after upload, followed by a success popup (OP-02); Part List Export Excel sheet "Upload" is the base file for Edit uploads (OP-02); allocation below or equal to Max Case/Day allowed and every destination row must have a destination (BR-16, OP-04).</t>
+          <t xml:space="preserve">Business decisions: Effective Start Date editable only while Candidate (BR-06 confirmed); Edit button kept next to the Part Number link (BR-07); ongoing period lists Active parts, past periods list every part (BR-12); "Validate file" = save after upload, followed by a success popup (OP-02); Part List Export Excel sheet "Upload" is the base file for Edit uploads (OP-02); upload template gets a status column: Candidate cannot be changed by upload, Active &lt;-&gt; Inactive can; allocation below or equal to Max Case/Day allowed and every destination row must have a destination (BR-16, OP-04).</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2395,102 +2395,119 @@
     <row r="23" ht="18.2" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>flag_add_edit</t>
+          <t xml:space="preserve">part_no</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Row marker: Add (new part) or Edit (already registered part)</t>
+          <t xml:space="preserve">Part Number</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Add: required. Edit: required.</t>
+          <t xml:space="preserve">Add: required. Edit: required.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18.2" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>part_no</t>
+          <t xml:space="preserve">minimum_mad</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Part Number</t>
+          <t xml:space="preserve">Minimum MAD</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Add: required. Edit: required.</t>
+          <t xml:space="preserve">Add: required. Edit: can be changed.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18.2" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>pcs_case</t>
+          <t xml:space="preserve">pcs_case</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Pieces per case</t>
+          <t xml:space="preserve">Pieces per case</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Add: required. Edit: can be changed.</t>
+          <t xml:space="preserve">Add: required. Edit: can be changed.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18.2" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>max_case_day</t>
+          <t xml:space="preserve">max_case_day</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Max Case/Day</t>
+          <t xml:space="preserve">Max Case/Day</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Add: required. Edit: can be changed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18.2" customHeight="1">
+          <t xml:space="preserve">Add: required. Edit: can be changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="46" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>minimum_mad</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Minimum MAD</t>
+          <t xml:space="preserve">Part status (Candidate / Active / Inactive)</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Add: required. Edit: can be changed.</t>
+          <t xml:space="preserve">Add: leave blank (a new part is always Candidate). Edit: a Candidate part keeps Candidate (validation rejects any other value); an Active part can be changed to Inactive and an Inactive part to Active; no part can be changed to Candidate.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="31.4" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>effective_start_date</t>
+          <t xml:space="preserve">flag_add_edit</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Effective date</t>
+          <t xml:space="preserve">Row marker: A = Add (new part), E = Edit (already registered part)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Add: required. Edit: can only be changed while the part status is still Candidate.</t>
+          <t xml:space="preserve">Add: required. Edit: required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="31.4" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">effective_start_date</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective Start Date (DD-Mon-YYYY)</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add: required. Edit: can only be changed while the part status is still Candidate.</t>
         </is>
       </c>
     </row>
@@ -7311,7 +7328,7 @@
       </c>
       <c r="B345" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The modal lists the template columns (flag_add_edit, part_no, pcs_case, max_case_day, minimum_mad, effective_start_date), the required columns for Add and Edit, a drag-and-drop area (.xlsx max 5 MB, max 5,000 rows), the "Download template .xlsx" link and the "Close" and "Validate file" buttons. After "Validate file" the modal closes and the popup "Saved successfully" appears (MSG-17).</t>
+          <t xml:space="preserve">The modal lists the template columns in the order of sheet "Upload" (part_no, minimum_mad, pcs_case, max_case_day, status, flag_add_edit, effective_start_date), the rules for Add and Edit, a drag-and-drop area (.xlsx max 5 MB, max 5,000 rows), the "Download template .xlsx" link and the "Close" and "Validate file" buttons. After "Validate file" the modal closes and the popup "Saved successfully" appears (MSG-17).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add UISS-Screen for Crossdock Master Setting - Part List
- UISS_Screen_PartList.xlsx (TMAP template): Gen Desc, 2 screen flows,
  13 screen layouts from the prototype, 56 items, 3 data map blocks,
  operation description, 13 display messages, 3 logging messages
- Spec and screenshots kept under deliverables/ for regeneration
- FSD Field Spec: restore the Export Excel rule (H7) that was overwritten
  with the Upload Excel text; Upload Excel rule moved to H6

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/FSD_Crossdock_Master_Setting.xlsx
+++ b/FSD_Crossdock_Master_Setting.xlsx
@@ -9511,7 +9511,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Opens the Upload Excel modal.</t>
+          <t xml:space="preserve">Opens the Upload Excel modal. "Validate file" in the modal validates and saves the uploaded file, then shows the success popup (OP-02).</t>
         </is>
       </c>
     </row>
@@ -9553,7 +9553,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opens the Upload Excel modal. "Validate file" in the modal validates and saves the uploaded file, then shows the success popup (OP-02).</t>
+          <t xml:space="preserve">Downloads Crossdock_Part_List_YYYYMMDD.xlsx: sheet "Part List" = rows of the active filter (information only); sheet "Upload" = every registered part pre-filled with flag E, the base file for Edit uploads (OP-02).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
All documents: project name Crossdock Optimization, author FID Rayhan
- UISS (6 workbooks): Project Name, Created By / Updated By and revision
  authors in the Revision sheet (header formulas on every sheet follow it)
- FSD (2 workbooks): Prepared by = FID Rayhan, cover subtitle starts with
  Crossdock Optimization
- UISS specs under deliverables/ updated to match

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/FSD_Crossdock_Master_Setting.xlsx
+++ b/FSD_Crossdock_Master_Setting.xlsx
@@ -1817,7 +1817,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>New Service Part System (NSP) · Master &gt; Crossdock Master Setting</t>
+          <t xml:space="preserve">Crossdock Optimization · New Service Part System (NSP) · Master &gt; Crossdock Master Setting</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,11 @@
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FID Rayhan</t>
+        </is>
+      </c>
       <c r="C13" s="9" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Revert FSD author/project change: the FSDs are no longer maintained
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/FSD_Crossdock_Master_Setting.xlsx
+++ b/FSD_Crossdock_Master_Setting.xlsx
@@ -1817,7 +1817,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crossdock Optimization · New Service Part System (NSP) · Master &gt; Crossdock Master Setting</t>
+          <t>New Service Part System (NSP) · Master &gt; Crossdock Master Setting</t>
         </is>
       </c>
     </row>
@@ -1896,11 +1896,7 @@
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FID Rayhan</t>
-        </is>
-      </c>
+      <c r="B13" s="9" t="n"/>
       <c r="C13" s="9" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">

</xml_diff>